<commit_message>
Ocultar claves de Supabase y añadir gunicorn
</commit_message>
<xml_diff>
--- a/data/inputs/ExcelCliente (3).xlsx
+++ b/data/inputs/ExcelCliente (3).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/525260a030f8d24b/TFG(proyecto)/proyecto/data/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{4C7F3A97-4671-40D2-B2FF-BBBE85474D1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{577A796D-9D21-545B-AF8A-08967A332F08}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{4C7F3A97-4671-40D2-B2FF-BBBE85474D1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E665A19E-4F78-4FC1-B250-E47E870D5F22}"/>
   <bookViews>
-    <workbookView xWindow="4044" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1464" yWindow="1464" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="damela hecha de google, con est" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="109">
   <si>
     <t>Nombre Restaurante</t>
   </si>
@@ -344,6 +344,9 @@
   </si>
   <si>
     <t>Gluten</t>
+  </si>
+  <si>
+    <t>Huevo</t>
   </si>
 </sst>
 </file>
@@ -706,7 +709,7 @@
         <v>19</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>20</v>
+        <v>108</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>